<commit_message>
Update Excel: quadratic function + neural net from fast.ai Lesson 3
</commit_message>
<xml_diff>
--- a/neuronales_netz.xlsx
+++ b/neuronales_netz.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neuronales Netz" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Quadratische Funktion" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Neuronales Netz" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,10 +28,17 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -42,12 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -68,12 +76,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -450,193 +460,587 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>x (Input)</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
+          <t>Quadratische Funktion: y = ax² + bx + c</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Parameter:</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>y (Richtig)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Vorhersage
-=x*w+b</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ReLU
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>y (Vorhersage)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Loss (B-C)²</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>-3</v>
+      </c>
+      <c r="B7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <f>$B$4*A7^2+$C$4*A7+$D$4</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>(B7-C7)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>-2</v>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <f>$B$4*A8^2+$C$4*A8+$D$4</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>(B8-C8)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <f>$B$4*A9^2+$C$4*A9+$D$4</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>(B9-C9)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>0</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <f>$B$4*A10^2+$C$4*A10+$D$4</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>(B10-C10)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <f>$B$4*A11^2+$C$4*A11+$D$4</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>(B11-C11)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12">
+        <f>$B$4*A12^2+$C$4*A12+$D$4</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>(B12-C12)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13">
+        <f>$B$4*A13^2+$C$4*A13+$D$4</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>(B13-C13)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Gesamt Loss:</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>AVERAGE(D7:D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Ziel: Ändere a, b, c bis Loss = 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Lösung: a=1, b=0, c=0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Neuronales Netz = Addition zweier ReLU Funktionen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Wie Jeremy Howard erklärt: Zwei Regressionsmodelle + ReLU = Neuronales Netz</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Parameter Linie 1:</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>w1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>b1</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Parameter Linie 2:</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>w2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>b2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>y (Richtig)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Linie 1
+=w1*x+b1</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>ReLU1
 =MAX(0,C)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Linie 2
+=w2*x+b2</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>ReLU2
+=MAX(0,E)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Netz
+=ReLU1+ReLU2</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Loss
-=(B-D)²</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+=(B-G)²</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-3</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <f>$B$6*A9+$C$6</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>MAX(0,C9)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>$F$6*A9+$G$6</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>MAX(0,E9)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>D9+F9</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>(B9-G9)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>-2</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <f>$B$6*A10+$C$6</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>MAX(0,C10)</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>$F$6*A10+$G$6</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>MAX(0,E10)</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>D10+F10</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>(B10-G10)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <f>$B$6*A11+$C$6</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>MAX(0,C11)</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>$F$6*A11+$G$6</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>MAX(0,E11)</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>D11+F11</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>(B11-G11)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>0</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <f>$B$6*A12+$C$6</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>MAX(0,C12)</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>$F$6*A12+$G$6</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>MAX(0,E12)</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>D12+F12</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>(B12-G12)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <f>$B$6*A13+$C$6</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>MAX(0,C13)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>$F$6*A13+$G$6</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>MAX(0,E13)</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>D13+F13</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>(B13-G13)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
         <v>2</v>
       </c>
-      <c r="C2">
-        <f>A2*$H$2+$H$3</f>
-        <v/>
-      </c>
-      <c r="D2">
-        <f>MAX(0,C2)</f>
-        <v/>
-      </c>
-      <c r="E2">
-        <f>(B2-D2)^2</f>
-        <v/>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Gewicht (w):</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="B14" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <f>A3*$H$2+$H$3</f>
-        <v/>
-      </c>
-      <c r="D3">
-        <f>MAX(0,C3)</f>
-        <v/>
-      </c>
-      <c r="E3">
-        <f>(B3-D3)^2</f>
-        <v/>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Bias (b):</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="C14">
+        <f>$B$6*A14+$C$6</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>MAX(0,C14)</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>$F$6*A14+$G$6</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>MAX(0,E14)</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>D14+F14</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>(B14-G14)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C4">
-        <f>A4*$H$2+$H$3</f>
-        <v/>
-      </c>
-      <c r="D4">
-        <f>MAX(0,C4)</f>
-        <v/>
-      </c>
-      <c r="E4">
-        <f>(B4-D4)^2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="n">
-        <v>8</v>
-      </c>
-      <c r="C5">
-        <f>A5*$H$2+$H$3</f>
-        <v/>
-      </c>
-      <c r="D5">
-        <f>MAX(0,C5)</f>
-        <v/>
-      </c>
-      <c r="E5">
-        <f>(B5-D5)^2</f>
-        <v/>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <f>$B$6*A15+$C$6</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>MAX(0,C15)</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>$F$6*A15+$G$6</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>MAX(0,E15)</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>D15+F15</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>(B15-G15)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Gesamt Loss:</t>
         </is>
       </c>
-      <c r="H5" s="4">
-        <f>AVERAGE(E2:E6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C6">
-        <f>A6*$H$2+$H$3</f>
-        <v/>
-      </c>
-      <c r="D6">
-        <f>MAX(0,C6)</f>
-        <v/>
-      </c>
-      <c r="E6">
-        <f>(B6-D6)^2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Anleitung:</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Ändere w (H2) und b (H3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>bis Gesamt Loss (H5) = 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Lösung: w=2, b=0</t>
+      <c r="B17" s="5">
+        <f>AVERAGE(H9:H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Das ist ein neuronales Netz mit 2 Neuronen!</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Ändere w1,b1,w2,b2 bis Loss = 0</t>
         </is>
       </c>
     </row>

</xml_diff>